<commit_message>
revision general de imports
</commit_message>
<xml_diff>
--- a/tests/coeficienteExtLineal1.xlsx
+++ b/tests/coeficienteExtLineal1.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12" uniqueCount="11">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="45" uniqueCount="39">
   <si>
     <t xml:space="preserve">DATOS DE Coeficiente de Extensibilidad Lineal</t>
   </si>
@@ -31,10 +31,10 @@
     <t xml:space="preserve">Rep</t>
   </si>
   <si>
-    <t xml:space="preserve">Longitud Inicial</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Diámetro de la muestra</t>
+    <t xml:space="preserve">Longitud Inicial (cm)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Diámetro de la muestra (mm)</t>
   </si>
   <si>
     <t xml:space="preserve">Fecha de Medición</t>
@@ -46,23 +46,109 @@
     <t xml:space="preserve">12.45</t>
   </si>
   <si>
+    <t xml:space="preserve">50.2</t>
+  </si>
+  <si>
     <t xml:space="preserve">12.38</t>
   </si>
   <si>
+    <t xml:space="preserve">50.1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">12.42</t>
+  </si>
+  <si>
+    <t xml:space="preserve">50.3</t>
+  </si>
+  <si>
     <t xml:space="preserve">13.02</t>
   </si>
   <si>
+    <t xml:space="preserve">51.0</t>
+  </si>
+  <si>
     <t xml:space="preserve">12.97</t>
+  </si>
+  <si>
+    <t xml:space="preserve">50.8</t>
+  </si>
+  <si>
+    <t xml:space="preserve">13.05</t>
+  </si>
+  <si>
+    <t xml:space="preserve">50.9</t>
+  </si>
+  <si>
+    <t xml:space="preserve">49.9</t>
+  </si>
+  <si>
+    <t xml:space="preserve">12.44</t>
+  </si>
+  <si>
+    <t xml:space="preserve">50.0</t>
+  </si>
+  <si>
+    <t xml:space="preserve">12.41</t>
+  </si>
+  <si>
+    <t xml:space="preserve">49.8</t>
+  </si>
+  <si>
+    <t xml:space="preserve">13.20</t>
+  </si>
+  <si>
+    <t xml:space="preserve">50.6</t>
+  </si>
+  <si>
+    <t xml:space="preserve">13.15</t>
+  </si>
+  <si>
+    <t xml:space="preserve">50.5</t>
+  </si>
+  <si>
+    <t xml:space="preserve">12.75</t>
+  </si>
+  <si>
+    <t xml:space="preserve">12.79</t>
+  </si>
+  <si>
+    <t xml:space="preserve">13.40</t>
+  </si>
+  <si>
+    <t xml:space="preserve">13.36</t>
+  </si>
+  <si>
+    <t xml:space="preserve">51.1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">12.60</t>
+  </si>
+  <si>
+    <t xml:space="preserve">49.7</t>
+  </si>
+  <si>
+    <t xml:space="preserve">12.63</t>
+  </si>
+  <si>
+    <t xml:space="preserve">13.10</t>
+  </si>
+  <si>
+    <t xml:space="preserve">50.4</t>
+  </si>
+  <si>
+    <t xml:space="preserve">13.07</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="1">
+  <numFmts count="3">
     <numFmt numFmtId="164" formatCode="General"/>
+    <numFmt numFmtId="165" formatCode="yyyy\-mm\-dd"/>
+    <numFmt numFmtId="166" formatCode="hh:mm:ss"/>
   </numFmts>
-  <fonts count="6">
+  <fonts count="7">
     <font>
       <sz val="10"/>
       <name val="Arial"/>
@@ -87,6 +173,13 @@
     <font>
       <b val="true"/>
       <sz val="14"/>
+      <name val="Arial"/>
+      <family val="2"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <b val="true"/>
+      <sz val="10"/>
       <name val="Arial"/>
       <family val="2"/>
       <charset val="1"/>
@@ -141,7 +234,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="13">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -158,8 +251,40 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
     <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
   </cellXfs>
@@ -182,37 +307,37 @@
         <a:srgbClr val="000000"/>
       </a:dk1>
       <a:lt1>
-        <a:srgbClr val="ffffff"/>
+        <a:srgbClr val="FFFFFF"/>
       </a:lt1>
       <a:dk2>
         <a:srgbClr val="000000"/>
       </a:dk2>
       <a:lt2>
-        <a:srgbClr val="ffffff"/>
+        <a:srgbClr val="FFFFFF"/>
       </a:lt2>
       <a:accent1>
-        <a:srgbClr val="18a303"/>
+        <a:srgbClr val="18A303"/>
       </a:accent1>
       <a:accent2>
-        <a:srgbClr val="0369a3"/>
+        <a:srgbClr val="0369A3"/>
       </a:accent2>
       <a:accent3>
-        <a:srgbClr val="a33e03"/>
+        <a:srgbClr val="A33E03"/>
       </a:accent3>
       <a:accent4>
-        <a:srgbClr val="8e03a3"/>
+        <a:srgbClr val="8E03A3"/>
       </a:accent4>
       <a:accent5>
-        <a:srgbClr val="c99c00"/>
+        <a:srgbClr val="C99C00"/>
       </a:accent5>
       <a:accent6>
-        <a:srgbClr val="c9211e"/>
+        <a:srgbClr val="C9211E"/>
       </a:accent6>
       <a:hlink>
-        <a:srgbClr val="0000ee"/>
+        <a:srgbClr val="0000EE"/>
       </a:hlink>
       <a:folHlink>
-        <a:srgbClr val="551a8b"/>
+        <a:srgbClr val="551A8B"/>
       </a:folHlink>
     </a:clrScheme>
     <a:fontScheme name="Office">
@@ -285,7 +410,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:N7"/>
+  <dimension ref="A1:N24"/>
   <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="19.2"/>
@@ -336,114 +461,424 @@
       <c r="F2" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="G2" s="4"/>
-      <c r="H2" s="4"/>
-      <c r="I2" s="4"/>
-      <c r="J2" s="4"/>
-      <c r="K2" s="4"/>
-      <c r="L2" s="4"/>
-      <c r="M2" s="4"/>
-      <c r="N2" s="4"/>
+      <c r="G2" s="5"/>
+      <c r="H2" s="5"/>
+      <c r="I2" s="5"/>
+      <c r="J2" s="5"/>
+      <c r="K2" s="5"/>
+      <c r="L2" s="5"/>
+      <c r="M2" s="5"/>
+      <c r="N2" s="5"/>
     </row>
     <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="B3" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="C3" s="1" t="s">
+      <c r="A3" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="B3" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="C3" s="6" t="s">
         <v>7</v>
       </c>
-      <c r="D3" s="1" t="n">
-        <v>226</v>
-      </c>
-      <c r="E3" s="1" t="n">
-        <v>215</v>
-      </c>
-      <c r="F3" s="1" t="n">
-        <v>209</v>
+      <c r="D3" s="6" t="s">
+        <v>8</v>
+      </c>
+      <c r="E3" s="7" t="n">
+        <v>45717</v>
+      </c>
+      <c r="F3" s="8" t="n">
+        <v>0.34375</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="B4" s="1" t="n">
-        <v>2</v>
-      </c>
-      <c r="C4" s="1" t="s">
+      <c r="A4" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="B4" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="C4" s="6" t="s">
+        <v>9</v>
+      </c>
+      <c r="D4" s="6" t="s">
+        <v>10</v>
+      </c>
+      <c r="E4" s="7" t="n">
+        <v>45717</v>
+      </c>
+      <c r="F4" s="8" t="n">
+        <v>0.364583333333333</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="B5" s="6" t="n">
+        <v>3</v>
+      </c>
+      <c r="C5" s="6" t="s">
+        <v>11</v>
+      </c>
+      <c r="D5" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="E5" s="7" t="n">
+        <v>45717</v>
+      </c>
+      <c r="F5" s="8" t="n">
+        <v>0.388888888888889</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="B6" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="C6" s="6" t="s">
+        <v>13</v>
+      </c>
+      <c r="D6" s="6" t="s">
+        <v>14</v>
+      </c>
+      <c r="E6" s="7" t="n">
+        <v>45718</v>
+      </c>
+      <c r="F6" s="8" t="n">
+        <v>0.381944444444444</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A7" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="B7" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="C7" s="6" t="s">
+        <v>15</v>
+      </c>
+      <c r="D7" s="6" t="s">
+        <v>16</v>
+      </c>
+      <c r="E7" s="7" t="n">
+        <v>45718</v>
+      </c>
+      <c r="F7" s="8" t="n">
+        <v>0.402777777777778</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A8" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="B8" s="6" t="n">
+        <v>3</v>
+      </c>
+      <c r="C8" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="D8" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="E8" s="7" t="n">
+        <v>45718</v>
+      </c>
+      <c r="F8" s="8" t="n">
+        <v>0.427083333333333</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A9" s="6" t="n">
+        <v>3</v>
+      </c>
+      <c r="B9" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="C9" s="6" t="s">
+        <v>9</v>
+      </c>
+      <c r="D9" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="E9" s="7" t="n">
+        <v>45719</v>
+      </c>
+      <c r="F9" s="8" t="n">
+        <v>0.430555555555556</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A10" s="6" t="n">
+        <v>3</v>
+      </c>
+      <c r="B10" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="C10" s="6" t="s">
+        <v>20</v>
+      </c>
+      <c r="D10" s="6" t="s">
+        <v>21</v>
+      </c>
+      <c r="E10" s="7" t="n">
+        <v>45719</v>
+      </c>
+      <c r="F10" s="8" t="n">
+        <v>0.451388888888889</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A11" s="6" t="n">
+        <v>3</v>
+      </c>
+      <c r="B11" s="6" t="n">
+        <v>3</v>
+      </c>
+      <c r="C11" s="6" t="s">
+        <v>22</v>
+      </c>
+      <c r="D11" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="E11" s="7" t="n">
+        <v>45719</v>
+      </c>
+      <c r="F11" s="8" t="n">
+        <v>0.475694444444444</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A12" s="6" t="n">
+        <v>4</v>
+      </c>
+      <c r="B12" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="C12" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="D12" s="6" t="s">
+        <v>25</v>
+      </c>
+      <c r="E12" s="7" t="n">
+        <v>45720</v>
+      </c>
+      <c r="F12" s="8" t="n">
+        <v>0.354166666666667</v>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A13" s="6" t="n">
+        <v>4</v>
+      </c>
+      <c r="B13" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="C13" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="D13" s="6" t="s">
+        <v>27</v>
+      </c>
+      <c r="E13" s="7" t="n">
+        <v>45720</v>
+      </c>
+      <c r="F13" s="8" t="n">
+        <v>0.378472222222222</v>
+      </c>
+    </row>
+    <row r="14" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A14" s="6" t="n">
+        <v>5</v>
+      </c>
+      <c r="B14" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="C14" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="D14" s="6" t="s">
         <v>8</v>
       </c>
-      <c r="D4" s="1" t="n">
-        <v>229</v>
-      </c>
-      <c r="E4" s="1" t="n">
-        <v>218</v>
-      </c>
-      <c r="F4" s="1" t="n">
-        <v>212</v>
-      </c>
-    </row>
-    <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="1" t="n">
-        <v>2</v>
-      </c>
-      <c r="B5" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="C5" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="D5" s="1" t="n">
-        <v>241</v>
-      </c>
-      <c r="E5" s="1" t="n">
-        <v>233</v>
-      </c>
-      <c r="F5" s="1" t="n">
-        <v>227</v>
-      </c>
-    </row>
-    <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="1" t="n">
-        <v>2</v>
-      </c>
-      <c r="B6" s="1" t="n">
-        <v>2</v>
-      </c>
-      <c r="C6" s="1" t="s">
+      <c r="E14" s="7" t="n">
+        <v>45721</v>
+      </c>
+      <c r="F14" s="8" t="n">
+        <v>0.385416666666667</v>
+      </c>
+    </row>
+    <row r="15" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A15" s="6" t="n">
+        <v>5</v>
+      </c>
+      <c r="B15" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="C15" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="D15" s="6" t="s">
         <v>10</v>
       </c>
-      <c r="D6" s="1" t="n">
-        <v>238</v>
-      </c>
-      <c r="E6" s="1" t="n">
-        <v>231</v>
-      </c>
-      <c r="F6" s="1" t="n">
-        <v>225</v>
-      </c>
-    </row>
-    <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A7" s="1" t="n">
-        <v>3</v>
-      </c>
-      <c r="B7" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="C7" s="1" t="s">
+      <c r="E15" s="7" t="n">
+        <v>45721</v>
+      </c>
+      <c r="F15" s="8" t="n">
+        <v>0.40625</v>
+      </c>
+    </row>
+    <row r="16" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A16" s="6" t="n">
+        <v>6</v>
+      </c>
+      <c r="B16" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="C16" s="6" t="s">
+        <v>30</v>
+      </c>
+      <c r="D16" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="E16" s="7" t="n">
+        <v>45722</v>
+      </c>
+      <c r="F16" s="8" t="n">
+        <v>0.347222222222222</v>
+      </c>
+    </row>
+    <row r="17" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A17" s="6" t="n">
+        <v>6</v>
+      </c>
+      <c r="B17" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="C17" s="6" t="s">
+        <v>31</v>
+      </c>
+      <c r="D17" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="E17" s="7" t="n">
+        <v>45722</v>
+      </c>
+      <c r="F17" s="8" t="n">
+        <v>0.371527777777778</v>
+      </c>
+    </row>
+    <row r="18" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A18" s="6" t="n">
+        <v>7</v>
+      </c>
+      <c r="B18" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="C18" s="6" t="s">
+        <v>33</v>
+      </c>
+      <c r="D18" s="6" t="s">
+        <v>34</v>
+      </c>
+      <c r="E18" s="7" t="n">
+        <v>45723</v>
+      </c>
+      <c r="F18" s="8" t="n">
+        <v>0.423611111111111</v>
+      </c>
+    </row>
+    <row r="19" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A19" s="6" t="n">
+        <v>7</v>
+      </c>
+      <c r="B19" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="C19" s="6" t="s">
+        <v>35</v>
+      </c>
+      <c r="D19" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="E19" s="7" t="n">
+        <v>45723</v>
+      </c>
+      <c r="F19" s="8" t="n">
+        <v>0.444444444444444</v>
+      </c>
+      <c r="G19" s="9"/>
+      <c r="H19" s="9"/>
+    </row>
+    <row r="20" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A20" s="6" t="n">
         <v>8</v>
       </c>
-      <c r="D7" s="1" t="n">
-        <v>229</v>
-      </c>
-      <c r="E7" s="1" t="n">
-        <v>218</v>
-      </c>
-      <c r="F7" s="1" t="n">
-        <v>212</v>
-      </c>
+      <c r="B20" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="C20" s="6" t="s">
+        <v>36</v>
+      </c>
+      <c r="D20" s="6" t="s">
+        <v>37</v>
+      </c>
+      <c r="E20" s="7" t="n">
+        <v>45724</v>
+      </c>
+      <c r="F20" s="8" t="n">
+        <v>0.375</v>
+      </c>
+      <c r="G20" s="10"/>
+      <c r="H20" s="11"/>
+    </row>
+    <row r="21" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A21" s="6" t="n">
+        <v>8</v>
+      </c>
+      <c r="B21" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="C21" s="6" t="s">
+        <v>38</v>
+      </c>
+      <c r="D21" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="E21" s="7" t="n">
+        <v>45724</v>
+      </c>
+      <c r="F21" s="8" t="n">
+        <v>0.395833333333333</v>
+      </c>
+      <c r="G21" s="10"/>
+      <c r="H21" s="11"/>
+    </row>
+    <row r="22" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="C22" s="12"/>
+      <c r="D22" s="12"/>
+      <c r="E22" s="12"/>
+      <c r="F22" s="12"/>
+      <c r="G22" s="10"/>
+      <c r="H22" s="11"/>
+    </row>
+    <row r="23" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="C23" s="12"/>
+      <c r="D23" s="12"/>
+      <c r="E23" s="12"/>
+      <c r="F23" s="12"/>
+      <c r="G23" s="10"/>
+      <c r="H23" s="11"/>
+    </row>
+    <row r="24" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="C24" s="12"/>
+      <c r="D24" s="12"/>
+      <c r="E24" s="12"/>
+      <c r="F24" s="12"/>
+      <c r="G24" s="10"/>
+      <c r="H24" s="11"/>
     </row>
   </sheetData>
   <mergeCells count="1">

</xml_diff>